<commit_message>
added 2026 round 6 results
</commit_message>
<xml_diff>
--- a/bio/player_bio.xlsx
+++ b/bio/player_bio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matevass/Documents/Programming/R/darts-statistics/bio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E4218B-6053-7548-AD28-8F4064440B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6DB93C-71EF-AB44-9DA9-6A0657628E4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
   <si>
     <t>Player</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>Bellini - Samba de Janeiro</t>
+  </si>
+  <si>
+    <t>26g Red Dragon Razor Edge</t>
   </si>
 </sst>
 </file>
@@ -722,7 +725,7 @@
         <v>44</v>
       </c>
       <c r="H4" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1005,7 +1008,7 @@
         <v>9</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="H15" s="6">
         <v>2</v>

</xml_diff>